<commit_message>
Multi-period reconciliation engine matching a bank statement against a general-ledger cash extract across four passes, with rule-based exception classification, completeness controls, and a SQL ledger that carries unresolved items forward between months, ages them, and proves nothing was lost via a rollforward control.
</commit_message>
<xml_diff>
--- a/output/reconciliation_report_jun2026.xlsx
+++ b/output/reconciliation_report_jun2026.xlsx
@@ -12,8 +12,10 @@
     <sheet name="Matched — Exact" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Matched — Timing" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Matched — Tolerance" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Bank Statement (source)" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="GL Extract (source)" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Open Items (aged)" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Rollforward" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Bank Statement (source)" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="GL Extract (source)" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -122,7 +124,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -153,6 +155,7 @@
     <xf numFmtId="167" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -656,7 +659,7 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="16">
@@ -666,7 +669,7 @@
         </is>
       </c>
       <c r="B16" s="9" t="n">
-        <v>120539.59</v>
+        <v>120539.94</v>
       </c>
     </row>
     <row r="18">
@@ -876,61 +879,61 @@
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">  add: bank charges not booked</t>
+          <t xml:space="preserve">  add: pass-3 amount residuals (pending write-off JE)</t>
         </is>
       </c>
       <c r="B39" s="9" t="n">
-        <v>-607.4400000000001</v>
+        <v>-0.35</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">  add: interest not booked (net)</t>
+          <t xml:space="preserve">  add: bank charges not booked</t>
         </is>
       </c>
       <c r="B40" s="9" t="n">
-        <v>-397.21</v>
+        <v>-607.4400000000001</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">  add: NSF returned deposits not booked</t>
+          <t xml:space="preserve">  add: interest not booked (net)</t>
         </is>
       </c>
       <c r="B41" s="9" t="n">
-        <v>-3875.4</v>
+        <v>-397.21</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">  add: unidentified bank items (pending ID)</t>
+          <t xml:space="preserve">  add: NSF returned deposits not booked</t>
         </is>
       </c>
       <c r="B42" s="9" t="n">
-        <v>890</v>
+        <v>-3875.4</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">  add back: duplicate postings to reverse</t>
+          <t xml:space="preserve">  add: unidentified bank items (pending ID)</t>
         </is>
       </c>
       <c r="B43" s="9" t="n">
-        <v>10230.18</v>
+        <v>890</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">  add: pass-3 amount residuals (pending write-off JE)</t>
+          <t xml:space="preserve">  add back: duplicate postings to reverse</t>
         </is>
       </c>
       <c r="B44" s="9" t="n">
-        <v>-0.35</v>
+        <v>10230.18</v>
       </c>
     </row>
     <row r="45">
@@ -972,7 +975,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J22"/>
+  <dimension ref="A1:J23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1843,6 +1846,46 @@
       </c>
       <c r="J22" s="24" t="n">
         <v>128</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>Residual</t>
+        </is>
+      </c>
+      <c r="C23" s="27" t="n">
+        <v>46203</v>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>Pass-3 amount residuals across matched pairs</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr"/>
+      <c r="F23" s="9" t="n">
+        <v>-0.35</v>
+      </c>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>RESIDUAL</t>
+        </is>
+      </c>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t>Pass-3 amount residuals — pending write-off JE</t>
+        </is>
+      </c>
+      <c r="I23" s="4" t="inlineStr">
+        <is>
+          <t>Book JE: write off the rounding difference to 6900 Misc Expense</t>
+        </is>
+      </c>
+      <c r="J23" s="4" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -7423,6 +7466,1049 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00BF8F00"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Open reconciling items at June 2026 close</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Every item still open, whichever period raised it, aged from its own transaction date. Flagged items need action, not just carrying.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Age bucket</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Items</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Exposure</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Flagged</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>0-30 days</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="C5" s="9" t="n">
+        <v>25153.12</v>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Origin period</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Doc/Ref</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>Age (days)</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>Bucket</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>Flag</t>
+        </is>
+      </c>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>Escalated</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="B8" s="27" t="n">
+        <v>46174</v>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Region of Halton — invoice payment</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>CHQ#1042</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="n">
+        <v>-10230.18</v>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>DUPLICATE</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="n">
+        <v>29</v>
+      </c>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>0-30</t>
+        </is>
+      </c>
+      <c r="I8" s="4" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="J8" s="4" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="B9" s="27" t="n">
+        <v>46185</v>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Cogeco underground build — change order</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>REF41002</t>
+        </is>
+      </c>
+      <c r="E9" s="9" t="n">
+        <v>9406.58</v>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>DEP_NOT_CREDITED</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>0-30</t>
+        </is>
+      </c>
+      <c r="I9" s="4" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="J9" s="4" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="B10" s="27" t="n">
+        <v>46191</v>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>NSF RETURNED ITEM FEE</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>NSF-0618</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="n">
+        <v>-48</v>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>BANK_CHARGE</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>0-30</t>
+        </is>
+      </c>
+      <c r="I10" s="4" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="J10" s="4" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="B11" s="27" t="n">
+        <v>46192</v>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>RETURNED ITEM NSF CUSTOMER CHQ 5521</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>RET-0619</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="n">
+        <v>-3875.4</v>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>NSF_RETURN</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>0-30</t>
+        </is>
+      </c>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="J11" s="4" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="B12" s="27" t="n">
+        <v>46195</v>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>MERCHANT PROCESSING FEE MONERIS</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>MER-0622</t>
+        </is>
+      </c>
+      <c r="E12" s="9" t="n">
+        <v>-389.44</v>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>BANK_CHARGE</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>0-30</t>
+        </is>
+      </c>
+      <c r="I12" s="4" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="J12" s="4" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="B13" s="27" t="n">
+        <v>46198</v>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>PRE-AUTH DEBIT UNKNOWN ORIG 7719</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>PAD-7719</t>
+        </is>
+      </c>
+      <c r="E13" s="9" t="n">
+        <v>-1260</v>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>UNID_DEBIT</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>0-30</t>
+        </is>
+      </c>
+      <c r="I13" s="4" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="J13" s="4" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="B14" s="27" t="n">
+        <v>46199</v>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Ditch Witch of Ontario — parts invoice</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>CHQ#1079</t>
+        </is>
+      </c>
+      <c r="E14" s="9" t="n">
+        <v>-7412.66</v>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>OS_CHECK</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>0-30</t>
+        </is>
+      </c>
+      <c r="I14" s="4" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="J14" s="4" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="B15" s="27" t="n">
+        <v>46199</v>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>E-TRANSFER RECEIVED T4X99A</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>ETR-T4X99A</t>
+        </is>
+      </c>
+      <c r="E15" s="9" t="n">
+        <v>2150</v>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>UNID_CREDIT</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>0-30</t>
+        </is>
+      </c>
+      <c r="I15" s="4" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="J15" s="4" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="B16" s="27" t="n">
+        <v>46202</v>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Vermeer Canada — drill head rebuild</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>CHQ#1080</t>
+        </is>
+      </c>
+      <c r="E16" s="9" t="n">
+        <v>-15890.23</v>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>OS_CHECK</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>0-30</t>
+        </is>
+      </c>
+      <c r="I16" s="4" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="J16" s="4" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="B17" s="27" t="n">
+        <v>46202</v>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Region of Halton — road permit fees</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>CHQ#1081</t>
+        </is>
+      </c>
+      <c r="E17" s="9" t="n">
+        <v>-2340.55</v>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>OS_CHECK</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>0-30</t>
+        </is>
+      </c>
+      <c r="I17" s="4" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="J17" s="4" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="B18" s="27" t="n">
+        <v>46202</v>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Enterprise Fleet Mgmt — vehicle lease unit 3</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>REF40990</t>
+        </is>
+      </c>
+      <c r="E18" s="9" t="n">
+        <v>-1286.43</v>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>PMT_IN_TRANSIT</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H18" s="4" t="inlineStr">
+        <is>
+          <t>0-30</t>
+        </is>
+      </c>
+      <c r="I18" s="4" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="J18" s="4" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="B19" s="27" t="n">
+        <v>46203</v>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Rogers Communications — progress billing</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>REF40947</t>
+        </is>
+      </c>
+      <c r="E19" s="9" t="n">
+        <v>48310.77</v>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>DIT</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" s="4" t="inlineStr">
+        <is>
+          <t>0-30</t>
+        </is>
+      </c>
+      <c r="I19" s="4" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="J19" s="4" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="B20" s="27" t="n">
+        <v>46203</v>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Cogeco underground build</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>REF40957</t>
+        </is>
+      </c>
+      <c r="E20" s="9" t="n">
+        <v>12764.31</v>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>DIT</t>
+        </is>
+      </c>
+      <c r="G20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" s="4" t="inlineStr">
+        <is>
+          <t>0-30</t>
+        </is>
+      </c>
+      <c r="I20" s="4" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="J20" s="4" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="B21" s="27" t="n">
+        <v>46203</v>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Brandt Tractor Ltd — service invoice</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>CHQ#1082</t>
+        </is>
+      </c>
+      <c r="E21" s="9" t="n">
+        <v>-4178.09</v>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>OS_CHECK</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>0-30</t>
+        </is>
+      </c>
+      <c r="I21" s="4" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="J21" s="4" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="B22" s="27" t="n">
+        <v>46203</v>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>INTEREST ON OPERATING LINE OF CREDIT</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>LOC-INT-JUN</t>
+        </is>
+      </c>
+      <c r="E22" s="9" t="n">
+        <v>-612.08</v>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>INTEREST_EXP</t>
+        </is>
+      </c>
+      <c r="G22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" s="4" t="inlineStr">
+        <is>
+          <t>0-30</t>
+        </is>
+      </c>
+      <c r="I22" s="4" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="J22" s="4" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="B23" s="27" t="n">
+        <v>46203</v>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>INTEREST EARNED</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>INT-JUN</t>
+        </is>
+      </c>
+      <c r="E23" s="9" t="n">
+        <v>214.87</v>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>INTEREST_INC</t>
+        </is>
+      </c>
+      <c r="G23" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t>0-30</t>
+        </is>
+      </c>
+      <c r="I23" s="4" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="J23" s="4" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="B24" s="27" t="n">
+        <v>46203</v>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>MONTHLY ACCOUNT FEE</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>SVC-JUN</t>
+        </is>
+      </c>
+      <c r="E24" s="9" t="n">
+        <v>-125</v>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>BANK_CHARGE</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" s="4" t="inlineStr">
+        <is>
+          <t>0-30</t>
+        </is>
+      </c>
+      <c r="I24" s="4" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="J24" s="4" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="B25" s="27" t="n">
+        <v>46203</v>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>SERVICE CHARGE - WIRE PAYMENT</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>WIRE-FEE</t>
+        </is>
+      </c>
+      <c r="E25" s="9" t="n">
+        <v>-45</v>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>BANK_CHARGE</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" s="4" t="inlineStr">
+        <is>
+          <t>0-30</t>
+        </is>
+      </c>
+      <c r="I25" s="4" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="J25" s="4" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="B26" s="27" t="n">
+        <v>46203</v>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>RESIDUAL</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr"/>
+      <c r="E26" s="9" t="n">
+        <v>-0.35</v>
+      </c>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t>RESIDUAL</t>
+        </is>
+      </c>
+      <c r="G26" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" s="4" t="inlineStr">
+        <is>
+          <t>0-30</t>
+        </is>
+      </c>
+      <c r="I26" s="4" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="J26" s="4" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="002F5597"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Reconciling items — rollforward</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>open at start + raised − cleared − written off = open at end. One period's closing items are the next one's opening items.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Period</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Open at start</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Raised</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Cleared</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Written off</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Open at end</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Exposure at end</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="G5" s="9" t="n">
+        <v>25153.12</v>
+      </c>
+      <c r="H5" s="28" t="inlineStr">
+        <is>
+          <t>BALANCED</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>No breaks: every period balances and rolls into the next.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="00808080"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -9749,7 +10835,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00808080"/>

</xml_diff>